<commit_message>
Deploy IG - 17a8f9eeed2c8342f235fc97278c0fefc1c89335 17a8f9eeed2c8342f235fc97278c0fefc1c89335
</commit_message>
<xml_diff>
--- a/StructureDefinition-ph-core-observation.xlsx
+++ b/StructureDefinition-ph-core-observation.xlsx
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-04-15T02:57:51+00:00</t>
+    <t>2026-04-22T03:27:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -516,7 +516,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(CarePlan|4.0.1|DeviceRequest|4.0.1|ImmunizationRecommendation|4.0.1|MedicationRequest|4.0.1|NutritionOrder|4.0.1|ServiceRequest|4.0.1)
+    <t xml:space="preserve">Reference(CarePlan|DeviceRequest|ImmunizationRecommendation|MedicationRequest|NutritionOrder|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-serviceRequest)
 </t>
   </si>
   <si>
@@ -545,7 +545,7 @@
 </t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(MedicationAdministration|4.0.1|MedicationDispense|4.0.1|MedicationStatement|4.0.1|Procedure|4.0.1|Immunization|4.0.1|ImagingStudy|4.0.1)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-medicationadministration|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-medicationdispense|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-medicationstatement|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-procedure|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-immunization|ImagingStudy)
 </t>
   </si>
   <si>
@@ -788,7 +788,7 @@
     <t>Observation.subject</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-patient)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-patient|Group|Device|Location)
 </t>
   </si>
   <si>
@@ -933,7 +933,7 @@
     <t>Observation.performer</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Practitioner|4.0.1|PractitionerRole|4.0.1|Organization|4.0.1|CareTeam|4.0.1|Patient|4.0.1|RelatedPerson|4.0.1)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-practitioner|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-practitionerrole|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-organization|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-patient|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-relatedperson|CareTeam)
 </t>
   </si>
   <si>
@@ -1482,7 +1482,7 @@
     <t>Observation.hasMember</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(Observation|4.0.1|QuestionnaireResponse|4.0.1|MolecularSequence|4.0.1)
+    <t xml:space="preserve">Reference(http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-observation|Observation|QuestionnaireResponse|MolecularSequence)
 </t>
   </si>
   <si>
@@ -1504,7 +1504,7 @@
     <t>Observation.derivedFrom</t>
   </si>
   <si>
-    <t xml:space="preserve">Reference(DocumentReference|4.0.1|ImagingStudy|4.0.1|Media|4.0.1|QuestionnaireResponse|4.0.1|Observation|4.0.1|MolecularSequence|4.0.1)
+    <t xml:space="preserve">Reference(DocumentReference|ImagingStudy|Media|QuestionnaireResponse|http://doh.gov.ph/fhir/ph-core/StructureDefinition/ph-core-observation|Observation|MolecularSequence)
 </t>
   </si>
   <si>
@@ -1993,7 +1993,7 @@
     <col min="8" max="8" width="13.953125" customWidth="true" bestFit="true"/>
     <col min="9" max="9" width="11.3671875" customWidth="true" bestFit="true"/>
     <col min="10" max="10" width="20.703125" customWidth="true" bestFit="true"/>
-    <col min="11" max="11" width="122.43359375" customWidth="true" bestFit="true"/>
+    <col min="11" max="11" width="255.0" customWidth="true" bestFit="true"/>
     <col min="12" max="12" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="13" max="13" width="100.703125" customWidth="true" bestFit="true"/>
     <col min="14" max="14" width="100.703125" customWidth="true" bestFit="true"/>

</xml_diff>